<commit_message>
Samsung all-SKU file: 13 more titles from retailer search
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Samsung_ALL_1561_titles.xlsx
+++ b/Samsung_ALL_1561_titles.xlsx
@@ -17719,48 +17719,54 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B339" s="2" t="inlineStr">
+      <c r="A339" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B339" s="3" t="inlineStr">
         <is>
           <t>6003-001449</t>
         </is>
       </c>
-      <c r="C339" s="2" t="n"/>
-      <c r="D339" s="2" t="n"/>
-      <c r="E339" s="2" t="n"/>
-      <c r="F339" s="2" t="inlineStr">
+      <c r="C339" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Taptype Screw - 6003-001449</t>
+        </is>
+      </c>
+      <c r="D339" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Taptype Screw - 6003-001449 | OEM Part</t>
+        </is>
+      </c>
+      <c r="E339" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F339" s="3" t="inlineStr">
         <is>
           <t>6003-001449</t>
         </is>
       </c>
-      <c r="G339" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H339" s="2" t="n"/>
-      <c r="I339" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J339" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K339" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Taptype Screw - 6003-001449</t>
-        </is>
-      </c>
-      <c r="L339" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED from part-number family, not confirmed for this exact part: 6003 series = taptype screws (14 of 15 confirmed). pass2 searched, no exact hit</t>
+      <c r="G339" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="H339" s="3" t="n"/>
+      <c r="I339" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J339" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="K339" s="3" t="n"/>
+      <c r="L339" s="3" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). INFERRED from part-number family, not confirmed for this exact part: 6003 series = taptype screws (14 of 15 confirmed). pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -23349,48 +23355,52 @@
       </c>
     </row>
     <row r="450">
-      <c r="A450" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B450" s="2" t="inlineStr">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
         <is>
           <t>BA96-07808A</t>
         </is>
       </c>
-      <c r="C450" s="2" t="n"/>
-      <c r="D450" s="2" t="n"/>
-      <c r="E450" s="2" t="n"/>
-      <c r="F450" s="2" t="inlineStr">
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Webcam - BA96-07808A</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Webcam - BA96-07808A | OEM Part</t>
+        </is>
+      </c>
+      <c r="E450" t="n">
+        <v>46</v>
+      </c>
+      <c r="F450" t="inlineStr">
         <is>
           <t>ba96-07808a</t>
         </is>
       </c>
-      <c r="G450" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H450" s="2" t="n"/>
-      <c r="I450" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J450" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K450" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop LCD Assembly - BA96-07808A</t>
-        </is>
-      </c>
-      <c r="L450" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED from part-number family, not confirmed for this exact part: BA96 series = laptop LCD assemblies (24 confirmed). searched, no exact hit</t>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>High (exact part number confirmed)</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). INFERRED from part-number family, not confirmed for this exact part: BA96 series = laptop LCD assemblies (24 confirmed). searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -28056,48 +28066,52 @@
       </c>
     </row>
     <row r="542">
-      <c r="A542" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B542" s="2" t="inlineStr">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
         <is>
           <t>BN39-02415A</t>
         </is>
       </c>
-      <c r="C542" s="2" t="n"/>
-      <c r="D542" s="2" t="n"/>
-      <c r="E542" s="2" t="n"/>
-      <c r="F542" s="2" t="inlineStr">
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Samsung TV Lead Connector Sub Assembly - BN39-02415A</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Samsung TV Lead Connector Sub Assembly - BN39-02415A</t>
+        </is>
+      </c>
+      <c r="E542" t="n">
+        <v>52</v>
+      </c>
+      <c r="F542" t="inlineStr">
         <is>
           <t>bn39-02415a</t>
         </is>
       </c>
-      <c r="G542" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H542" s="2" t="n"/>
-      <c r="I542" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J542" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K542" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02415A</t>
-        </is>
-      </c>
-      <c r="L542" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED from part-number family, not confirmed for this exact part: BN39 series = TV cables/leads (97 confirmed, all cable/connector types). searched, no exact hit</t>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="I542" t="inlineStr">
+        <is>
+          <t>High (exact part number confirmed)</t>
+        </is>
+      </c>
+      <c r="J542" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="L542" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). INFERRED from part-number family, not confirmed for this exact part: BN39 series = TV cables/leads (97 confirmed, all cable/connector types). searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -33402,48 +33416,52 @@
       </c>
     </row>
     <row r="648">
-      <c r="A648" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B648" s="2" t="inlineStr">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
         <is>
           <t>AH81-17358A</t>
         </is>
       </c>
-      <c r="C648" s="2" t="n"/>
-      <c r="D648" s="2" t="n"/>
-      <c r="E648" s="2" t="n"/>
-      <c r="F648" s="2" t="inlineStr">
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Wireless Module (TX) - AH81-17358A</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Wireless Module (TX) - AH81-17358A</t>
+        </is>
+      </c>
+      <c r="E648" t="n">
+        <v>51</v>
+      </c>
+      <c r="F648" t="inlineStr">
         <is>
           <t>ah81-17358a</t>
         </is>
       </c>
-      <c r="G648" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H648" s="2" t="n"/>
-      <c r="I648" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J648" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K648" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-17358A</t>
-        </is>
-      </c>
-      <c r="L648" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="I648" t="inlineStr">
+        <is>
+          <t>High (exact part number confirmed)</t>
+        </is>
+      </c>
+      <c r="J648" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="L648" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -39791,48 +39809,52 @@
       </c>
     </row>
     <row r="775">
-      <c r="A775" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B775" s="2" t="inlineStr">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
         <is>
           <t>AH44-00315A</t>
         </is>
       </c>
-      <c r="C775" s="2" t="n"/>
-      <c r="D775" s="2" t="n"/>
-      <c r="E775" s="2" t="n"/>
-      <c r="F775" s="2" t="inlineStr">
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>Samsung Home Theater Power Supply Board - AH44-00315A</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Samsung Home Theater Power Supply Board - AH44-00315A</t>
+        </is>
+      </c>
+      <c r="E775" t="n">
+        <v>53</v>
+      </c>
+      <c r="F775" t="inlineStr">
         <is>
           <t>ah44-00315a</t>
         </is>
       </c>
-      <c r="G775" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H775" s="2" t="n"/>
-      <c r="I775" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J775" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K775" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH44-00315A</t>
-        </is>
-      </c>
-      <c r="L775" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="G775" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="I775" t="inlineStr">
+        <is>
+          <t>High (exact part number confirmed)</t>
+        </is>
+      </c>
+      <c r="J775" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="L775" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -43337,48 +43359,52 @@
       </c>
     </row>
     <row r="846">
-      <c r="A846" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B846" s="2" t="inlineStr">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
         <is>
           <t>BA97-12799A</t>
         </is>
       </c>
-      <c r="C846" s="2" t="n"/>
-      <c r="D846" s="2" t="n"/>
-      <c r="E846" s="2" t="n"/>
-      <c r="F846" s="2" t="inlineStr">
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Front Top Case Assembly - BA97-12799A</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Front Top Case Assembly - BA97-12799A</t>
+        </is>
+      </c>
+      <c r="E846" t="n">
+        <v>52</v>
+      </c>
+      <c r="F846" t="inlineStr">
         <is>
           <t>ba97-12799a</t>
         </is>
       </c>
-      <c r="G846" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H846" s="2" t="n"/>
-      <c r="I846" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J846" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K846" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop Replacement Part - BA97-12799A</t>
-        </is>
-      </c>
-      <c r="L846" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="I846" t="inlineStr">
+        <is>
+          <t>High (exact part number confirmed)</t>
+        </is>
+      </c>
+      <c r="J846" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="L846" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -50648,48 +50674,54 @@
       </c>
     </row>
     <row r="991">
-      <c r="A991" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B991" s="2" t="inlineStr">
+      <c r="A991" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B991" s="3" t="inlineStr">
         <is>
           <t>BN39-02471A</t>
         </is>
       </c>
-      <c r="C991" s="2" t="n"/>
-      <c r="D991" s="2" t="n"/>
-      <c r="E991" s="2" t="n"/>
-      <c r="F991" s="2" t="inlineStr">
+      <c r="C991" s="3" t="inlineStr">
+        <is>
+          <t>Samsung TV One Connect Cable - BN39-02471A</t>
+        </is>
+      </c>
+      <c r="D991" s="3" t="inlineStr">
+        <is>
+          <t>Samsung TV One Connect Cable - BN39-02471A | OEM Part</t>
+        </is>
+      </c>
+      <c r="E991" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="F991" s="3" t="inlineStr">
         <is>
           <t>bn39-02471a</t>
         </is>
       </c>
-      <c r="G991" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H991" s="2" t="n"/>
-      <c r="I991" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J991" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K991" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02471A</t>
-        </is>
-      </c>
-      <c r="L991" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED from part-number family, not confirmed for this exact part: BN39 series = TV cables/leads (97 confirmed, all cable/connector types). searched, no exact hit</t>
+      <c r="G991" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="H991" s="3" t="n"/>
+      <c r="I991" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J991" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="K991" s="3" t="n"/>
+      <c r="L991" s="3" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). INFERRED from part-number family, not confirmed for this exact part: BN39 series = TV cables/leads (97 confirmed, all cable/connector types). searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -51231,48 +51263,52 @@
       </c>
     </row>
     <row r="1003">
-      <c r="A1003" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1003" s="2" t="inlineStr">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
         <is>
           <t>6003-001917</t>
         </is>
       </c>
-      <c r="C1003" s="2" t="n"/>
-      <c r="D1003" s="2" t="n"/>
-      <c r="E1003" s="2" t="n"/>
-      <c r="F1003" s="2" t="inlineStr">
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Samsung Taptype Screw (SWRCH22A) - 6003-001917</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>Samsung Taptype Screw (SWRCH22A) - 6003-001917 | OEM Part</t>
+        </is>
+      </c>
+      <c r="E1003" t="n">
+        <v>57</v>
+      </c>
+      <c r="F1003" t="inlineStr">
         <is>
           <t>6003-001917</t>
         </is>
       </c>
-      <c r="G1003" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H1003" s="2" t="n"/>
-      <c r="I1003" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J1003" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K1003" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Taptype Screw - 6003-001917</t>
-        </is>
-      </c>
-      <c r="L1003" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED from part-number family, not confirmed for this exact part: 6003 series = taptype screws (14 of 15 confirmed). searched, no exact hit</t>
+      <c r="G1003" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="I1003" t="inlineStr">
+        <is>
+          <t>High (exact part number confirmed)</t>
+        </is>
+      </c>
+      <c r="J1003" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="L1003" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). INFERRED from part-number family, not confirmed for this exact part: 6003 series = taptype screws (14 of 15 confirmed). searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -51377,48 +51413,52 @@
       </c>
     </row>
     <row r="1006">
-      <c r="A1006" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1006" s="2" t="inlineStr">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
         <is>
           <t>6006-001170</t>
         </is>
       </c>
-      <c r="C1006" s="2" t="n"/>
-      <c r="D1006" s="2" t="n"/>
-      <c r="E1006" s="2" t="n"/>
-      <c r="F1006" s="2" t="inlineStr">
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Samsung Tapping Screw (M4 x 10 mm, White) - 6006-001170</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>Samsung Tapping Screw (M4 x 10 mm, White) - 6006-001170</t>
+        </is>
+      </c>
+      <c r="E1006" t="n">
+        <v>55</v>
+      </c>
+      <c r="F1006" t="inlineStr">
         <is>
           <t>6006-001170</t>
         </is>
       </c>
-      <c r="G1006" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H1006" s="2" t="n"/>
-      <c r="I1006" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J1006" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K1006" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 6006-001170</t>
-        </is>
-      </c>
-      <c r="L1006" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="G1006" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="I1006" t="inlineStr">
+        <is>
+          <t>High (exact part number confirmed)</t>
+        </is>
+      </c>
+      <c r="J1006" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="L1006" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -56981,48 +57021,52 @@
       </c>
     </row>
     <row r="1117">
-      <c r="A1117" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1117" s="2" t="inlineStr">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
         <is>
           <t>AH81-14796A</t>
         </is>
       </c>
-      <c r="C1117" s="2" t="n"/>
-      <c r="D1117" s="2" t="n"/>
-      <c r="E1117" s="2" t="n"/>
-      <c r="F1117" s="2" t="inlineStr">
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Samsung Subwoofer (PS-WA65D) - AH81-14796A</t>
+        </is>
+      </c>
+      <c r="D1117" t="inlineStr">
+        <is>
+          <t>Samsung Subwoofer (PS-WA65D) - AH81-14796A | OEM Part</t>
+        </is>
+      </c>
+      <c r="E1117" t="n">
+        <v>53</v>
+      </c>
+      <c r="F1117" t="inlineStr">
         <is>
           <t>ah81-14796a</t>
         </is>
       </c>
-      <c r="G1117" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H1117" s="2" t="n"/>
-      <c r="I1117" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J1117" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K1117" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-14796A</t>
-        </is>
-      </c>
-      <c r="L1117" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit (summary text mentioned /es/products/ah81-14796a but no returned link carried the PN in its title)</t>
+      <c r="G1117" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="I1117" t="inlineStr">
+        <is>
+          <t>High (exact part number confirmed)</t>
+        </is>
+      </c>
+      <c r="J1117" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="L1117" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit (summary text mentioned /es/products/ah81-14796a but no returned link carried the PN in its title)</t>
         </is>
       </c>
     </row>
@@ -62073,48 +62117,52 @@
       </c>
     </row>
     <row r="1217">
-      <c r="A1217" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1217" s="2" t="inlineStr">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
         <is>
           <t>4709-003180</t>
         </is>
       </c>
-      <c r="C1217" s="2" t="n"/>
-      <c r="D1217" s="2" t="n"/>
-      <c r="E1217" s="2" t="n"/>
-      <c r="F1217" s="2" t="inlineStr">
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>Samsung Microwave Wireless LAN Module (CCAR210R) - 4709-003180</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>Samsung Microwave Wireless LAN Module (CCAR210R) - 4709-003180</t>
+        </is>
+      </c>
+      <c r="E1217" t="n">
+        <v>62</v>
+      </c>
+      <c r="F1217" t="inlineStr">
         <is>
           <t>4709-003180</t>
         </is>
       </c>
-      <c r="G1217" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H1217" s="2" t="n"/>
-      <c r="I1217" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J1217" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K1217" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 4709-003180</t>
-        </is>
-      </c>
-      <c r="L1217" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="G1217" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="I1217" t="inlineStr">
+        <is>
+          <t>High (exact part number confirmed)</t>
+        </is>
+      </c>
+      <c r="J1217" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="L1217" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -66274,48 +66322,52 @@
       </c>
     </row>
     <row r="1300">
-      <c r="A1300" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1300" s="2" t="inlineStr">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
         <is>
           <t>AH39-00474A</t>
         </is>
       </c>
-      <c r="C1300" s="2" t="n"/>
-      <c r="D1300" s="2" t="n"/>
-      <c r="E1300" s="2" t="n"/>
-      <c r="F1300" s="2" t="inlineStr">
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>Samsung USB Cable - AH39-00474A</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>Samsung USB Cable - AH39-00474A | OEM Part</t>
+        </is>
+      </c>
+      <c r="E1300" t="n">
+        <v>42</v>
+      </c>
+      <c r="F1300" t="inlineStr">
         <is>
           <t>ah39-00474a</t>
         </is>
       </c>
-      <c r="G1300" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H1300" s="2" t="n"/>
-      <c r="I1300" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J1300" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K1300" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH39-00474A</t>
-        </is>
-      </c>
-      <c r="L1300" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="G1300" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="I1300" t="inlineStr">
+        <is>
+          <t>High (exact part number confirmed)</t>
+        </is>
+      </c>
+      <c r="J1300" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="L1300" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -73744,48 +73796,54 @@
       </c>
     </row>
     <row r="1446">
-      <c r="A1446" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1446" s="2" t="inlineStr">
+      <c r="A1446" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1446" s="3" t="inlineStr">
         <is>
           <t>6001-002903</t>
         </is>
       </c>
-      <c r="C1446" s="2" t="n"/>
-      <c r="D1446" s="2" t="n"/>
-      <c r="E1446" s="2" t="n"/>
-      <c r="F1446" s="2" t="inlineStr">
+      <c r="C1446" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Machine Screw (M3 x 8 mm, Black) - 6001-002903</t>
+        </is>
+      </c>
+      <c r="D1446" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Machine Screw (M3 x 8 mm, Black) - 6001-002903</t>
+        </is>
+      </c>
+      <c r="E1446" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="F1446" s="3" t="inlineStr">
         <is>
           <t>6001-002903</t>
         </is>
       </c>
-      <c r="G1446" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="H1446" s="2" t="n"/>
-      <c r="I1446" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="J1446" s="2" t="inlineStr">
-        <is>
-          <t>OPEN - needs real title</t>
-        </is>
-      </c>
-      <c r="K1446" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Machine Screw - 6001-002903</t>
-        </is>
-      </c>
-      <c r="L1446" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED from part-number family, not confirmed for this exact part: 6001 series = machine screws (11 of 15 confirmed parts in this series). searched, no exact hit</t>
+      <c r="G1446" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (page not found by search)</t>
+        </is>
+      </c>
+      <c r="H1446" s="3" t="n"/>
+      <c r="I1446" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J1446" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="K1446" s="3" t="n"/>
+      <c r="L1446" s="3" t="inlineStr">
+        <is>
+          <t>Pass 5 retailer-site match (exact part number in listing title). INFERRED from part-number family, not confirmed for this exact part: 6001 series = machine screws (11 of 15 confirmed parts in this series). searched, no exact hit</t>
         </is>
       </c>
     </row>

</xml_diff>